<commit_message>
feat: harden reimbursement workflow
</commit_message>
<xml_diff>
--- a/plugins/xiaohongshu-reimbursement-workflow/skills/xiaohongshu-reimbursement-workflow/assets/templates/xiaohongshu/current-detail.xlsx
+++ b/plugins/xiaohongshu-reimbursement-workflow/skills/xiaohongshu-reimbursement-workflow/assets/templates/xiaohongshu/current-detail.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="7">
+  <x:numFmts count="11">
     <x:numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <x:numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
@@ -17,6 +17,10 @@
     <x:numFmt numFmtId="176" formatCode="0.000"/>
     <x:numFmt numFmtId="177" formatCode="mm\-dd"/>
     <x:numFmt numFmtId="178" formatCode="0.0"/>
+    <x:numFmt numFmtId="210" formatCode="0"/>
+    <x:numFmt numFmtId="211" formatCode="0.0"/>
+    <x:numFmt numFmtId="212" formatCode="0.00"/>
+    <x:numFmt numFmtId="213" formatCode="0.000"/>
   </x:numFmts>
   <x:fonts count="35">
     <x:font>
@@ -810,7 +814,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="75">
+  <x:cellXfs count="93">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -827,16 +831,16 @@
     <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="176" fontId="4" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="1" fontId="4" fillId="5" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="210" fontId="4" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="4" fillId="5" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="176" fontId="4" fillId="5" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="176" fontId="4" fillId="6" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="210" fontId="4" fillId="6" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -851,7 +855,7 @@
     <x:xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="176" fontId="8" fillId="4" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="210" fontId="8" fillId="4" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="177" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -860,10 +864,10 @@
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="1" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="210" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="1" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="210" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1027,6 +1031,60 @@
     <x:xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="4" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="4" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="4" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="4" fillId="5" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="4" fillId="5" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="4" fillId="5" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="4" fillId="6" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="4" fillId="6" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="4" fillId="6" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="4" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="8" fillId="4" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="8" fillId="4" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="9" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="50">
@@ -1457,6 +1515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1470,80 +1529,86 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;分类&gt;｜&lt;主期间&gt;</t>
+          <t>&lt;主期间&gt; 本次报销明细（按人员分类）</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">本次报销明细（按人员分类）</t>
+          <t>主期：&lt;主期间&gt;｜补报：&lt;补报摘要&gt;｜对公已付不实报单列</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">实报合计</t>
+          <t>主期实报</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">对公已付不实报</t>
+          <t>补报（&lt;笔数&gt;笔）</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">费用合计</t>
+          <t>实报合计</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="C4" s="7"/>
-      <c r="E4" s="9"/>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;补报说明&gt;</t>
+          <t>对公已付不实报：&lt;金额&gt;</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;无截图说明&gt;</t>
+          <t>费用合计：&lt;金额&gt;</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">日期</t>
+          <t>日期</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">支出明细</t>
+          <t>支出明细</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">支出金额</t>
+          <t>单笔金额</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">费用组合计</t>
+          <t>费用组合计</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">费用分类</t>
+          <t>备注 / 分类</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">结算方式</t>
+          <t>报销属性</t>
         </is>
       </c>
     </row>

</xml_diff>